<commit_message>
Improve Naive Bayes engine and activation visualization
</commit_message>
<xml_diff>
--- a/data/Data 15 Hari.xlsx
+++ b/data/Data 15 Hari.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\source\repos\Earthquake_Volcano (2)\Earthquake_Volcano\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laygenda surya putra\Documents\JOKI\gempavulkanik\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A87D9D-DE19-4497-81F5-98B79035389D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2BF9E4-3200-4856-BF53-4E06C8736EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="28">
   <si>
     <t>Tanggal</t>
   </si>
@@ -143,13 +143,19 @@
 3 kali gempa Tektonik Jauh
 1 kali gempa Tremor Menerus</t>
   </si>
+  <si>
+    <t>Gunung Kelud, Kediri</t>
+  </si>
+  <si>
+    <t>4 kali gempa Tektonik Jauh</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -211,7 +217,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,13 +520,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" customWidth="1"/>
+    <col min="1" max="1" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -546,7 +552,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>46000.949305555558</v>
       </c>
@@ -572,7 +578,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>46000.949305555558</v>
       </c>
@@ -598,7 +604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>46000.969444444447</v>
       </c>
@@ -624,7 +630,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>46000.969444444447</v>
       </c>
@@ -650,7 +656,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>46002.140277777777</v>
       </c>
@@ -676,7 +682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>46002.140277777777</v>
       </c>
@@ -702,7 +708,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>46002.918055555558</v>
       </c>
@@ -728,7 +734,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>46002.918055555558</v>
       </c>
@@ -754,7 +760,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>46003.140277777777</v>
       </c>
@@ -780,7 +786,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>46003.140277777777</v>
       </c>
@@ -806,7 +812,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>46003.22152777778</v>
       </c>
@@ -832,7 +838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>46003.22152777778</v>
       </c>
@@ -858,7 +864,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>46003.236805555563</v>
       </c>
@@ -884,7 +890,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>46003.236805555563</v>
       </c>
@@ -910,7 +916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>46003.761111111111</v>
       </c>
@@ -936,7 +942,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>46003.761111111111</v>
       </c>
@@ -962,7 +968,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>46004.627083333333</v>
       </c>
@@ -988,7 +994,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>46004.627083333333</v>
       </c>
@@ -1014,7 +1020,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>46004.629861111112</v>
       </c>
@@ -1040,7 +1046,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>46004.629861111112</v>
       </c>
@@ -1066,7 +1072,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>46004.977083333331</v>
       </c>
@@ -1092,7 +1098,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>46004.977083333331</v>
       </c>
@@ -1118,7 +1124,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>46004.995833333327</v>
       </c>
@@ -1144,7 +1150,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>46004.995833333327</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>46006.008333333331</v>
       </c>
@@ -1196,7 +1202,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>46006.008333333331</v>
       </c>
@@ -1222,7 +1228,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>46006.482638888891</v>
       </c>
@@ -1248,7 +1254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>46006.482638888891</v>
       </c>
@@ -1274,7 +1280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>46006.86041666667</v>
       </c>
@@ -1300,7 +1306,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>46006.86041666667</v>
       </c>
@@ -1326,29 +1332,81 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
+        <v>46174.895833333336</v>
+      </c>
+      <c r="B32">
+        <v>-7.91</v>
+      </c>
+      <c r="C32">
+        <v>112.32</v>
+      </c>
+      <c r="D32">
+        <v>2.4</v>
+      </c>
+      <c r="E32">
+        <v>101</v>
+      </c>
+      <c r="F32" t="s">
+        <v>26</v>
+      </c>
+      <c r="G32" t="s">
+        <v>27</v>
+      </c>
+      <c r="H32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
         <v>46189.35833333333</v>
       </c>
-      <c r="B32">
+      <c r="B33">
         <v>-7.89</v>
       </c>
-      <c r="C32">
+      <c r="C33">
         <v>114.34</v>
       </c>
-      <c r="D32">
+      <c r="D33">
         <v>2.7</v>
       </c>
-      <c r="E32">
+      <c r="E33">
         <v>4</v>
       </c>
-      <c r="F32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" t="s">
+      <c r="F33" t="s">
+        <v>11</v>
+      </c>
+      <c r="G33" t="s">
         <v>25</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>46208.15</v>
+      </c>
+      <c r="B34">
+        <v>-7.7</v>
+      </c>
+      <c r="C34">
+        <v>112.42</v>
+      </c>
+      <c r="D34">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E34">
+        <v>264</v>
+      </c>
+      <c r="F34" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" t="s">
+        <v>27</v>
+      </c>
+      <c r="H34" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>